<commit_message>
medina report + comments
</commit_message>
<xml_diff>
--- a/data collection/robot-variances.xlsx
+++ b/data collection/robot-variances.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://epflch-my.sharepoint.com/personal/medina_colabrese_epfl_ch/Documents/0 Mobile Robots/EPFL-BOMR-Project/data collection/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="8_{3A290D08-C5B6-4EB9-8BA6-6E071B2BC3F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6FD6D50F-63CA-4278-9A35-2B8CFD746E93}"/>
+  <xr:revisionPtr revIDLastSave="74" documentId="8_{3A290D08-C5B6-4EB9-8BA6-6E071B2BC3F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{683E20DD-0AC0-4BAC-B4EA-3D860BD4B0EA}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{D2DFFF4B-EF3D-44C8-A022-9334171DD194}"/>
+    <workbookView xWindow="5508" yWindow="-17388" windowWidth="30936" windowHeight="16776" xr2:uid="{D2DFFF4B-EF3D-44C8-A022-9334171DD194}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,14 +18,14 @@
   <definedNames>
     <definedName name="_xlchart.v1.0" hidden="1">Sheet1!$B$1</definedName>
     <definedName name="_xlchart.v1.1" hidden="1">Sheet1!$B$2:$B$228</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Sheet1!$A$1</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Sheet1!$A$2:$A$228</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Sheet1!$E$1</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">Sheet1!$E$2:$E$345</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">Sheet1!$E$1</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">Sheet1!$E$2:$E$345</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">Sheet1!$C$1</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">Sheet1!$C$2:$C$345</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Sheet1!$C$1</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Sheet1!$C$2:$C$345</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Sheet1!$A$1</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Sheet1!$A$2:$A$228</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">Sheet1!$C$1</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">Sheet1!$C$2:$C$345</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">Sheet1!$E$1</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">Sheet1!$E$2:$E$345</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -140,7 +140,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.3</cx:f>
+        <cx:f>_xlchart.v1.5</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -178,7 +178,7 @@
         <cx:series layoutId="clusteredColumn" uniqueId="{9515C7F9-73E1-4743-9E7F-753D37FE1E05}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.2</cx:f>
+              <cx:f>_xlchart.v1.4</cx:f>
               <cx:v>velocity error</cx:v>
             </cx:txData>
           </cx:tx>
@@ -190,10 +190,67 @@
       </cx:plotAreaRegion>
       <cx:axis id="0">
         <cx:catScaling gapWidth="0"/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Error [mm/s]</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                </a:rPr>
+                <a:t>Error [mm/s]</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
         <cx:tickLabels/>
+        <cx:numFmt formatCode="#,##0.00" sourceLinked="0"/>
       </cx:axis>
       <cx:axis id="1">
         <cx:valScaling/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Count</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                </a:rPr>
+                <a:t>Count</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
         <cx:majorGridlines/>
         <cx:tickLabels/>
       </cx:axis>
@@ -257,10 +314,67 @@
       </cx:plotAreaRegion>
       <cx:axis id="0">
         <cx:catScaling gapWidth="0"/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Error [mm]</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                </a:rPr>
+                <a:t>Error [mm]</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
         <cx:tickLabels/>
+        <cx:numFmt formatCode="#,##0.00" sourceLinked="0"/>
       </cx:axis>
       <cx:axis id="1">
         <cx:valScaling/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Count</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                </a:rPr>
+                <a:t>Count</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
         <cx:majorGridlines/>
         <cx:tickLabels/>
       </cx:axis>
@@ -274,7 +388,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.9</cx:f>
+        <cx:f>_xlchart.v1.3</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -312,7 +426,7 @@
         <cx:series layoutId="clusteredColumn" uniqueId="{75AA03BB-D29C-4A2F-B1D6-6349D2E28DE0}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.8</cx:f>
+              <cx:f>_xlchart.v1.2</cx:f>
               <cx:v>angular velocity error</cx:v>
             </cx:txData>
           </cx:tx>
@@ -324,10 +438,67 @@
       </cx:plotAreaRegion>
       <cx:axis id="0">
         <cx:catScaling gapWidth="0"/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Error [rad/s]</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                </a:rPr>
+                <a:t>Error [rad/s]</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
         <cx:tickLabels/>
+        <cx:numFmt formatCode="#,##0.00" sourceLinked="0"/>
       </cx:axis>
       <cx:axis id="1">
         <cx:valScaling/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Count</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                </a:rPr>
+                <a:t>Count</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
         <cx:majorGridlines/>
         <cx:tickLabels/>
       </cx:axis>
@@ -341,7 +512,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.7</cx:f>
+        <cx:f>_xlchart.v1.9</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -379,7 +550,7 @@
         <cx:series layoutId="clusteredColumn" uniqueId="{BC319B88-B6E2-4740-8193-0F3AC2538996}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.6</cx:f>
+              <cx:f>_xlchart.v1.8</cx:f>
               <cx:v>theta error adjusted</cx:v>
             </cx:txData>
           </cx:tx>
@@ -393,10 +564,67 @@
       </cx:plotAreaRegion>
       <cx:axis id="0">
         <cx:catScaling gapWidth="0"/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Error [rad]</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                </a:rPr>
+                <a:t>Error [rad]</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
         <cx:tickLabels/>
+        <cx:numFmt formatCode="#,##0.00" sourceLinked="0"/>
       </cx:axis>
       <cx:axis id="1">
         <cx:valScaling/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Count</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                </a:rPr>
+                <a:t>Count</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
         <cx:majorGridlines/>
         <cx:tickLabels/>
       </cx:axis>
@@ -2602,15 +2830,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>388620</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>20955</xdr:rowOff>
+      <xdr:colOff>514350</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>125730</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>20955</xdr:rowOff>
+      <xdr:colOff>251460</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
@@ -2646,7 +2874,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="3589020" y="1849755"/>
+              <a:off x="5334000" y="4531995"/>
               <a:ext cx="4572000" cy="2743200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -2679,16 +2907,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>396240</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>62865</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>521970</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>97155</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>487680</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>62865</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>259080</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>97155</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
@@ -2724,7 +2952,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="8431530" y="1891665"/>
+              <a:off x="5341620" y="1743075"/>
               <a:ext cx="4572000" cy="2743200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -2757,16 +2985,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>363855</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>32385</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>268605</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>139065</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>100965</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>32385</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>360045</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>139065</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
@@ -2802,7 +3030,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="3564255" y="4787265"/>
+              <a:off x="9923145" y="4528185"/>
               <a:ext cx="4572000" cy="2743200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -2836,15 +3064,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>333375</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>55245</xdr:rowOff>
+      <xdr:colOff>287655</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>93345</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
-      <xdr:colOff>424815</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>55245</xdr:rowOff>
+      <xdr:colOff>379095</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>93345</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
@@ -2880,7 +3108,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="8368665" y="4810125"/>
+              <a:off x="9942195" y="1739265"/>
               <a:ext cx="4572000" cy="2743200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -3231,10 +3459,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4F7A6D9-B925-41B9-9B3E-9CCF80F7A001}">
-  <dimension ref="A1:H345"/>
+  <dimension ref="A1:W345"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="7" max="7" width="13.734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.20703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.26171875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.62890625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.62890625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.89453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -3271,7 +3503,7 @@
         <f>IF(D2&lt;-PI(), D2+2*PI(), D2)</f>
         <v>0.41044328295528598</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="H2">
@@ -3296,7 +3528,7 @@
         <f t="shared" ref="E3:E66" si="0">IF(D3&lt;-PI(), D3+2*PI(), D3)</f>
         <v>1.6951610061556543E-2</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="H3">
@@ -3321,7 +3553,7 @@
         <f t="shared" si="0"/>
         <v>-2.5163960939962298E-3</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="1" t="s">
         <v>4</v>
       </c>
       <c r="H4">
@@ -3346,7 +3578,7 @@
         <f t="shared" si="0"/>
         <v>-2.2933452385728501E-2</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="1" t="s">
         <v>7</v>
       </c>
       <c r="H5">
@@ -3552,7 +3784,7 @@
         <v>-1.6939861097120298E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A17">
         <v>-2.72000000000076E-2</v>
       </c>
@@ -3570,7 +3802,7 @@
         <v>-3.6181370556971099E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A18">
         <v>3.6367999999999898</v>
       </c>
@@ -3588,7 +3820,7 @@
         <v>-6.1060267868309204E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A19">
         <v>2.9039999999999901</v>
       </c>
@@ -3605,8 +3837,12 @@
         <f t="shared" si="0"/>
         <v>1.1245368965726799E-2</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="W19">
+        <f>4.48+0.364</f>
+        <v>4.8440000000000003</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A20">
         <v>2.9039999999999901</v>
       </c>
@@ -3623,8 +3859,12 @@
         <f t="shared" si="0"/>
         <v>-2.4190937729795001E-2</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="W20">
+        <f>4.48+0.213</f>
+        <v>4.6930000000000005</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A21">
         <v>7.30079999999999</v>
       </c>
@@ -3642,7 +3882,7 @@
         <v>1.7587777890630301E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A22">
         <v>7.30079999999999</v>
       </c>
@@ -3659,8 +3899,12 @@
         <f t="shared" si="0"/>
         <v>-7.35668780432741E-3</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="W22">
+        <f>0.00156+0.00051</f>
+        <v>2.0699999999999998E-3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A23">
         <v>7.30079999999999</v>
       </c>
@@ -3678,7 +3922,7 @@
         <v>-3.63366304828103E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A24">
         <v>7.30079999999999</v>
       </c>
@@ -3696,7 +3940,7 @@
         <v>-3.0942640169035998E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A25">
         <v>4.7359999999999998</v>
       </c>
@@ -3714,7 +3958,7 @@
         <v>1.37334898029339E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A26">
         <v>4.3696000000000002</v>
       </c>
@@ -3732,7 +3976,7 @@
         <v>-3.5414934045570001E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A27">
         <v>4.3696000000000002</v>
       </c>
@@ -3750,7 +3994,7 @@
         <v>3.0736104651687499E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A28">
         <v>1.8048</v>
       </c>
@@ -3768,7 +4012,7 @@
         <v>-2.76972132780272E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A29">
         <v>1.8048</v>
       </c>
@@ -3786,7 +4030,7 @@
         <v>-7.2946389692118898E-4</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A30">
         <v>0.339200000000005</v>
       </c>
@@ -3804,7 +4048,7 @@
         <v>4.5160425147349097E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A31">
         <v>-2.0424000000000002</v>
       </c>
@@ -3822,7 +4066,7 @@
         <v>-2.0337730364841201E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A32">
         <v>-2.0424000000000002</v>
       </c>

</xml_diff>